<commit_message>
feat(resource): intake FY2569 paper/waste/GHG Jan–Jul partials
Sync OneDrive Resource workbooks, extend extractors for waste/GHG, and publish PUBLISHABLE_PARTIAL dashboard JSON. Water/energy unchanged; fuel still empty. No progress/score inference.
</commit_message>
<xml_diff>
--- a/data/staging/source/1.5waste2026.xlsx
+++ b/data/staging/source/1.5waste2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://maejo365-my.sharepoint.com/personal/researchmju_mju_ac_th/Documents/RAE-Document-Center/07-GreenOffice/resource/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CD5792A3-5894-48DC-B796-602822E04CFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="8_{CD5792A3-5894-48DC-B796-602822E04CFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B004B6B1-4A8A-4AF2-9E88-9A4BBAFFAE01}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" tabRatio="498" xr2:uid="{34B2156F-77D1-47CB-857F-BB5C2E1BAEB5}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="52">
   <si>
     <t>แบบฟอร์ม 4.1(1)</t>
   </si>
@@ -50,7 +50,7 @@
     <t>รายการขยะ</t>
   </si>
   <si>
-    <t>ปริมาณ (ระบุหน่วยเป็น ก.ก. หรือ ลิตร ) ปี 2568</t>
+    <t>ปริมาณ (ระบุหน่วยเป็น ก.ก. หรือ ลิตร ) ปี 2569</t>
   </si>
   <si>
     <t>ม.ค.</t>
@@ -72,21 +72,6 @@
   </si>
   <si>
     <t>ก.ค.</t>
-  </si>
-  <si>
-    <t>ส.ค.</t>
-  </si>
-  <si>
-    <t>ก.ย.</t>
-  </si>
-  <si>
-    <t>ต.ค.</t>
-  </si>
-  <si>
-    <t>พ.ย.</t>
-  </si>
-  <si>
-    <t>ธ.ค.</t>
   </si>
   <si>
     <t>ขยะทั่วไป (ฝังกลบเท่านั้น)</t>
@@ -131,7 +116,7 @@
     <t>ขวดพลาสติก</t>
   </si>
   <si>
-    <t>ใบไม้</t>
+    <t>ใบไม้-กิ่งไม้</t>
   </si>
   <si>
     <t>เศษอาหาร</t>
@@ -150,6 +135,21 @@
   </si>
   <si>
     <t xml:space="preserve">ปริมาณ (ระบุหน่วยเป็น ก.ก. หรือ ลิตร ) </t>
+  </si>
+  <si>
+    <t>ส.ค.</t>
+  </si>
+  <si>
+    <t>ก.ย.</t>
+  </si>
+  <si>
+    <t>ต.ค.</t>
+  </si>
+  <si>
+    <t>พ.ย.</t>
+  </si>
+  <si>
+    <t>ธ.ค.</t>
   </si>
   <si>
     <t>ขยะทั่วไป</t>
@@ -216,10 +216,16 @@
     <t xml:space="preserve">%การนำขยะกลับมาใช้ใหม่รวม 6 เดือน = </t>
   </si>
   <si>
+    <t>ปริมาณ (ระบุหน่วยเป็น ก.ก. หรือ ลิตร ) ปี 2568</t>
+  </si>
+  <si>
     <t>ขยะทั่วไป (ฝังกลบ)</t>
   </si>
   <si>
     <t>%ขยะอันตราย</t>
+  </si>
+  <si>
+    <t>ใบไม้</t>
   </si>
   <si>
     <t>อาหาร</t>
@@ -227,19 +233,16 @@
   <si>
     <t>2. รายการขยะของแต่ละประเภทสามรถเพิ่มเติมหรือตัดออกได้ขึ้นอยู่กับขยะที่เกิดขึ้นของแต่ละสำนักงาน</t>
   </si>
-  <si>
-    <t>ปริมาณ (ระบุหน่วยเป็น ก.ก. หรือ ลิตร ) ปี 2569</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="187" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="188" formatCode="0.0%"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="17">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -326,12 +329,6 @@
       <color theme="0"/>
       <name val="Cordia New"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="16"/>
-      <color theme="1"/>
-      <name val="Tahoma"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -547,7 +544,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -641,10 +638,10 @@
     <xf numFmtId="9" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="188" fontId="4" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="188" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -761,10 +758,7 @@
     <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -785,8 +779,32 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="187" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -797,37 +815,13 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="ปกติ" xfId="0" builtinId="0"/>
-    <cellStyle name="เปอร์เซ็นต์" xfId="1" builtinId="5"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -845,7 +839,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="th-TH"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -890,7 +884,7 @@
             <c:strRef>
               <c:f>'ปริมาณขยะรายเดือน '!$B$3:$M$3</c:f>
               <c:strCache>
-                <c:ptCount val="12"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>ม.ค.</c:v>
                 </c:pt>
@@ -911,21 +905,6 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>ก.ค.</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>ส.ค.</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>ก.ย.</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>ต.ค.</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>พ.ย.</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>ธ.ค.</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -937,40 +916,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>370.6</c:v>
+                  <c:v>351.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>336.1</c:v>
+                  <c:v>514.4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>383.5</c:v>
+                  <c:v>527.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>359.8</c:v>
+                  <c:v>405</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>411.4</c:v>
+                  <c:v>450</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>420.9</c:v>
+                  <c:v>465</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>359.4</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>365.6</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>350.8</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>341.8</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>349.8</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>331.3</c:v>
+                  <c:v>480</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1008,7 +972,7 @@
             <c:strRef>
               <c:f>'ปริมาณขยะรายเดือน '!$B$3:$M$3</c:f>
               <c:strCache>
-                <c:ptCount val="12"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>ม.ค.</c:v>
                 </c:pt>
@@ -1029,21 +993,6 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>ก.ค.</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>ส.ค.</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>ก.ย.</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>ต.ค.</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>พ.ย.</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>ธ.ค.</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1055,40 +1004,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
+                  <c:v>1.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.3</c:v>
-                </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.3</c:v>
+                  <c:v>4.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.7</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>10.8</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.9</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.2</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>2.5</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1126,7 +1060,7 @@
             <c:strRef>
               <c:f>'ปริมาณขยะรายเดือน '!$B$3:$M$3</c:f>
               <c:strCache>
-                <c:ptCount val="12"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>ม.ค.</c:v>
                 </c:pt>
@@ -1147,21 +1081,6 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>ก.ค.</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>ส.ค.</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>ก.ย.</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>ต.ค.</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>พ.ย.</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>ธ.ค.</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1173,40 +1092,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>97.5</c:v>
+                  <c:v>99.399999999999991</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>81.8</c:v>
+                  <c:v>73.400000000000006</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>132.5</c:v>
+                  <c:v>171.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>103.6</c:v>
+                  <c:v>106.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>146.6</c:v>
+                  <c:v>83</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>106.69999999999999</c:v>
+                  <c:v>84</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>100.69999999999999</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>98.5</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>88.9</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>114.6</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>65.5</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>86.100000000000009</c:v>
+                  <c:v>69</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1421,7 +1325,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="th-TH"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1515,7 +1419,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>0.20828882717368083</c:v>
+                  <c:v>0.21971706454465073</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.19560019129603057</c:v>
@@ -1524,31 +1428,31 @@
                   <c:v>0.25663374007360062</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.22356495468277945</c:v>
+                  <c:v>0.2080078125</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.26052958947929628</c:v>
+                  <c:v>0.15485074626865672</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.19817979197622584</c:v>
+                  <c:v>0.14867256637168141</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.21796536796536797</c:v>
+                  <c:v>0.12477396021699819</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.21223874165050635</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.20163302336130645</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.24972760950098061</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.15771731278593787</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.20627695256348827</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1625,7 +1529,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>0.7917111728263192</c:v>
+                  <c:v>0.77763041556145007</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.80368244858919169</c:v>
@@ -1634,31 +1538,31 @@
                   <c:v>0.74278520240170454</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.77643504531722063</c:v>
+                  <c:v>0.791015625</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.73111782477341392</c:v>
+                  <c:v>0.83955223880597019</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.78176077265973254</c:v>
+                  <c:v>0.82300884955752207</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.77792207792207801</c:v>
+                  <c:v>0.86799276672694392</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.78776125834949362</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.79564527103651628</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.74482458051863154</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.84228268721406208</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.79372304743651168</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1740,7 +1644,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>2.6525198938992041E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>7.1736011477761829E-4</c:v>
@@ -1749,25 +1653,25 @@
                   <c:v>5.8105752469494478E-4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>9.765625E-4</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8.3525857472898542E-3</c:v>
+                  <c:v>5.597014925373134E-3</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2.0059435364041606E-2</c:v>
+                  <c:v>2.831858407079646E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.1125541125541128E-3</c:v>
+                  <c:v>7.2332730560578659E-3</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.7217056021773644E-3</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5.4478099803878842E-3</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
@@ -1929,7 +1833,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="th-TH"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2444,7 +2348,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="th-TH"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -3410,41 +3314,41 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFDF2539-117C-4C01-B345-CF6A43275F9F}">
   <dimension ref="A1:M22"/>
-  <sheetFormatPr defaultRowHeight="27.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="27.75"/>
   <cols>
     <col min="1" max="1" width="29.5703125" style="8" customWidth="1"/>
     <col min="2" max="13" width="7.7109375" style="9" customWidth="1"/>
     <col min="14" max="16384" width="9.140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" ht="25.5" customHeight="1">
       <c r="B1" s="8"/>
       <c r="K1" s="30"/>
       <c r="L1" s="9" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:13" s="29" customFormat="1" ht="26.25" x14ac:dyDescent="0.2">
-      <c r="A2" s="85" t="s">
+    <row r="2" spans="1:13" s="29" customFormat="1" ht="26.25">
+      <c r="A2" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="88" t="s">
-        <v>50</v>
-      </c>
-      <c r="C2" s="89"/>
-      <c r="D2" s="89"/>
-      <c r="E2" s="89"/>
-      <c r="F2" s="89"/>
-      <c r="G2" s="89"/>
-      <c r="H2" s="89"/>
-      <c r="I2" s="89"/>
-      <c r="J2" s="89"/>
-      <c r="K2" s="89"/>
-      <c r="L2" s="89"/>
-      <c r="M2" s="90"/>
+      <c r="B2" s="81" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="82"/>
+      <c r="D2" s="82"/>
+      <c r="E2" s="82"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="82"/>
+      <c r="H2" s="82"/>
+      <c r="I2" s="82"/>
+      <c r="J2" s="82"/>
+      <c r="K2" s="82"/>
+      <c r="L2" s="82"/>
+      <c r="M2" s="83"/>
     </row>
-    <row r="3" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="86"/>
+    <row r="3" spans="1:13" ht="21" customHeight="1">
+      <c r="A3" s="85"/>
       <c r="B3" s="54" t="s">
         <v>3</v>
       </c>
@@ -3466,66 +3370,46 @@
       <c r="H3" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
+    </row>
+    <row r="4" spans="1:13" ht="23.25" customHeight="1">
+      <c r="A4" s="67" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="15" t="s">
+      <c r="B4" s="63">
+        <v>351.8</v>
+      </c>
+      <c r="C4" s="63">
+        <v>514.4</v>
+      </c>
+      <c r="D4" s="63">
+        <v>527.5</v>
+      </c>
+      <c r="E4" s="63">
+        <v>405</v>
+      </c>
+      <c r="F4" s="63">
+        <v>450</v>
+      </c>
+      <c r="G4" s="63">
+        <v>465</v>
+      </c>
+      <c r="H4" s="68">
+        <v>480</v>
+      </c>
+      <c r="I4" s="69"/>
+      <c r="J4" s="69"/>
+      <c r="K4" s="69"/>
+      <c r="L4" s="69"/>
+      <c r="M4" s="69"/>
+    </row>
+    <row r="5" spans="1:13" ht="23.25" customHeight="1">
+      <c r="A5" s="48" t="s">
         <v>11</v>
-      </c>
-      <c r="K3" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="L3" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="M3" s="15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="67" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="63">
-        <v>370.6</v>
-      </c>
-      <c r="C4" s="63">
-        <v>336.1</v>
-      </c>
-      <c r="D4" s="63">
-        <v>383.5</v>
-      </c>
-      <c r="E4" s="63">
-        <v>359.8</v>
-      </c>
-      <c r="F4" s="63">
-        <v>411.4</v>
-      </c>
-      <c r="G4" s="63">
-        <v>420.9</v>
-      </c>
-      <c r="H4" s="68">
-        <v>359.4</v>
-      </c>
-      <c r="I4" s="69">
-        <v>365.6</v>
-      </c>
-      <c r="J4" s="69">
-        <v>350.8</v>
-      </c>
-      <c r="K4" s="69">
-        <v>341.8</v>
-      </c>
-      <c r="L4" s="69">
-        <v>349.8</v>
-      </c>
-      <c r="M4" s="69">
-        <v>331.3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="48" t="s">
-        <v>16</v>
       </c>
       <c r="B5" s="55"/>
       <c r="C5" s="55"/>
@@ -3540,308 +3424,233 @@
       <c r="L5" s="55"/>
       <c r="M5" s="55"/>
     </row>
-    <row r="6" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="23.25" customHeight="1">
       <c r="A6" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="57">
+        <v>4.5</v>
+      </c>
+      <c r="E6" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="57">
+        <v>1</v>
+      </c>
+      <c r="H6" s="56">
+        <v>1</v>
+      </c>
+      <c r="I6" s="55"/>
+      <c r="J6" s="55"/>
+      <c r="K6" s="55"/>
+      <c r="L6" s="55"/>
+      <c r="M6" s="55"/>
+    </row>
+    <row r="7" spans="1:13" ht="23.25" customHeight="1">
+      <c r="A7" s="49" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="57">
+        <v>5</v>
+      </c>
+      <c r="H7" s="56" t="s">
+        <v>13</v>
+      </c>
+      <c r="I7" s="55"/>
+      <c r="J7" s="55"/>
+      <c r="K7" s="55"/>
+      <c r="L7" s="55"/>
+      <c r="M7" s="55"/>
+    </row>
+    <row r="8" spans="1:13" ht="23.25" customHeight="1">
+      <c r="A8" s="50" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="56" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" s="55"/>
+      <c r="J8" s="55"/>
+      <c r="K8" s="55"/>
+      <c r="L8" s="55"/>
+      <c r="M8" s="55"/>
+    </row>
+    <row r="9" spans="1:13" ht="23.25" customHeight="1">
+      <c r="A9" s="50" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="56" t="s">
+        <v>13</v>
+      </c>
+      <c r="I9" s="55"/>
+      <c r="J9" s="55"/>
+      <c r="K9" s="55"/>
+      <c r="L9" s="55"/>
+      <c r="M9" s="55"/>
+    </row>
+    <row r="10" spans="1:13" s="79" customFormat="1" ht="51" customHeight="1">
+      <c r="A10" s="76" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="57" t="s">
+      <c r="B10" s="57">
+        <v>1.2</v>
+      </c>
+      <c r="C10" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="57">
+        <v>0.5</v>
+      </c>
+      <c r="F10" s="57">
+        <v>3</v>
+      </c>
+      <c r="G10" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="77" t="s">
+        <v>13</v>
+      </c>
+      <c r="I10" s="78"/>
+      <c r="J10" s="78"/>
+      <c r="K10" s="78"/>
+      <c r="L10" s="78"/>
+      <c r="M10" s="78"/>
+    </row>
+    <row r="11" spans="1:13" ht="23.25" customHeight="1">
+      <c r="A11" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="57">
-        <v>3.5</v>
-      </c>
-      <c r="G6" s="57">
-        <v>9.5</v>
-      </c>
-      <c r="H6" s="56" t="s">
-        <v>18</v>
-      </c>
-      <c r="I6" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="J6" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="K6" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="L6" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="M6" s="55" t="s">
-        <v>18</v>
-      </c>
+      <c r="B11" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="57">
+        <v>10</v>
+      </c>
+      <c r="H11" s="56">
+        <v>3</v>
+      </c>
+      <c r="I11" s="55"/>
+      <c r="J11" s="55"/>
+      <c r="K11" s="55"/>
+      <c r="L11" s="55"/>
+      <c r="M11" s="55"/>
     </row>
-    <row r="7" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="49" t="s">
+    <row r="12" spans="1:13" ht="23.25" customHeight="1">
+      <c r="A12" s="48" t="s">
         <v>19</v>
-      </c>
-      <c r="B7" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="G7" s="57">
-        <v>0.5</v>
-      </c>
-      <c r="H7" s="56" t="s">
-        <v>18</v>
-      </c>
-      <c r="I7" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="J7" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="K7" s="55">
-        <v>2.5</v>
-      </c>
-      <c r="L7" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="M7" s="55" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="50" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="73" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="G8" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="H8" s="56">
-        <v>0.7</v>
-      </c>
-      <c r="I8" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="J8" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="K8" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="L8" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="M8" s="55" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="50" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="H9" s="56" t="s">
-        <v>18</v>
-      </c>
-      <c r="I9" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="J9" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="K9" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="L9" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="M9" s="55" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" s="80" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="77" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="E10" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="F10" s="57">
-        <v>1.2</v>
-      </c>
-      <c r="G10" s="57">
-        <v>0.8</v>
-      </c>
-      <c r="H10" s="78">
-        <v>1.2</v>
-      </c>
-      <c r="I10" s="79" t="s">
-        <v>18</v>
-      </c>
-      <c r="J10" s="79">
-        <v>1.2</v>
-      </c>
-      <c r="K10" s="79" t="s">
-        <v>18</v>
-      </c>
-      <c r="L10" s="79" t="s">
-        <v>18</v>
-      </c>
-      <c r="M10" s="79" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="57">
-        <v>0.3</v>
-      </c>
-      <c r="D11" s="57">
-        <v>0.3</v>
-      </c>
-      <c r="E11" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="F11" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="G11" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="H11" s="56" t="s">
-        <v>18</v>
-      </c>
-      <c r="I11" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="J11" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="K11" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="L11" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="M11" s="55" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="48" t="s">
-        <v>24</v>
       </c>
       <c r="B12" s="58">
         <f>SUM(B6:B11)</f>
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="C12" s="58">
         <f t="shared" ref="C12:M12" si="0">SUM(C6:C11)</f>
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D12" s="58">
         <f t="shared" si="0"/>
-        <v>0.3</v>
+        <v>4.5</v>
       </c>
       <c r="E12" s="58">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F12" s="58">
         <f t="shared" si="0"/>
-        <v>4.7</v>
+        <v>3</v>
       </c>
       <c r="G12" s="58">
         <f t="shared" si="0"/>
-        <v>10.8</v>
+        <v>16</v>
       </c>
       <c r="H12" s="58">
         <f t="shared" si="0"/>
-        <v>1.9</v>
-      </c>
-      <c r="I12" s="58">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J12" s="58">
-        <f t="shared" si="0"/>
-        <v>1.2</v>
-      </c>
-      <c r="K12" s="58">
-        <f t="shared" si="0"/>
-        <v>2.5</v>
-      </c>
-      <c r="L12" s="58">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M12" s="58">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="I12" s="58"/>
+      <c r="J12" s="58"/>
+      <c r="K12" s="58"/>
+      <c r="L12" s="58"/>
+      <c r="M12" s="58"/>
     </row>
-    <row r="13" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" ht="23.25" customHeight="1">
       <c r="A13" s="52" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B13" s="59"/>
       <c r="C13" s="55"/>
@@ -3856,277 +3665,212 @@
       <c r="L13" s="55"/>
       <c r="M13" s="55"/>
     </row>
-    <row r="14" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" ht="23.25" customHeight="1">
       <c r="A14" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="57">
+        <v>35</v>
+      </c>
+      <c r="C14" s="57">
+        <v>7.1</v>
+      </c>
+      <c r="D14" s="57">
+        <v>65</v>
+      </c>
+      <c r="E14" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="56" t="s">
+        <v>13</v>
+      </c>
+      <c r="I14" s="55"/>
+      <c r="J14" s="55"/>
+      <c r="K14" s="55"/>
+      <c r="L14" s="55"/>
+      <c r="M14" s="55"/>
+    </row>
+    <row r="15" spans="1:13" ht="23.25" customHeight="1">
+      <c r="A15" s="51" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="57">
+        <v>12.8</v>
+      </c>
+      <c r="C15" s="57">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="D15" s="57">
+        <v>8</v>
+      </c>
+      <c r="E15" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" s="56" t="s">
+        <v>13</v>
+      </c>
+      <c r="I15" s="55"/>
+      <c r="J15" s="55"/>
+      <c r="K15" s="55"/>
+      <c r="L15" s="55"/>
+      <c r="M15" s="55"/>
+    </row>
+    <row r="16" spans="1:13" ht="23.25" customHeight="1">
+      <c r="A16" s="53" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="57">
+        <v>6.8</v>
+      </c>
+      <c r="C16" s="57">
+        <v>3.5</v>
+      </c>
+      <c r="D16" s="57">
+        <v>7</v>
+      </c>
+      <c r="E16" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H16" s="56" t="s">
+        <v>13</v>
+      </c>
+      <c r="I16" s="55"/>
+      <c r="J16" s="55"/>
+      <c r="K16" s="55"/>
+      <c r="L16" s="55"/>
+      <c r="M16" s="55"/>
+    </row>
+    <row r="17" spans="1:13" ht="23.25" customHeight="1">
+      <c r="A17" s="51" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="57">
+        <v>0</v>
+      </c>
+      <c r="C17" s="57">
+        <v>0</v>
+      </c>
+      <c r="D17" s="57">
+        <v>0</v>
+      </c>
+      <c r="E17" s="57">
+        <v>2</v>
+      </c>
+      <c r="F17" s="57">
+        <v>6</v>
+      </c>
+      <c r="G17" s="57">
+        <v>7</v>
+      </c>
+      <c r="H17" s="56" t="s">
+        <v>13</v>
+      </c>
+      <c r="I17" s="55"/>
+      <c r="J17" s="55"/>
+      <c r="K17" s="55"/>
+      <c r="L17" s="55"/>
+      <c r="M17" s="55"/>
+    </row>
+    <row r="18" spans="1:13" ht="23.25" customHeight="1">
+      <c r="A18" s="53" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="57">
+        <v>44.8</v>
+      </c>
+      <c r="C18" s="57">
+        <v>58.2</v>
+      </c>
+      <c r="D18" s="57">
+        <v>91.5</v>
+      </c>
+      <c r="E18" s="57">
+        <v>104.5</v>
+      </c>
+      <c r="F18" s="57">
+        <v>77</v>
+      </c>
+      <c r="G18" s="57">
+        <v>77</v>
+      </c>
+      <c r="H18" s="56">
+        <v>69</v>
+      </c>
+      <c r="I18" s="55"/>
+      <c r="J18" s="55"/>
+      <c r="K18" s="55"/>
+      <c r="L18" s="55"/>
+      <c r="M18" s="55"/>
+    </row>
+    <row r="19" spans="1:13" ht="55.5">
+      <c r="A19" s="64" t="s">
         <v>26</v>
-      </c>
-      <c r="B14" s="57">
-        <v>10.199999999999999</v>
-      </c>
-      <c r="C14" s="57">
-        <v>3.2</v>
-      </c>
-      <c r="D14" s="57">
-        <v>4.7</v>
-      </c>
-      <c r="E14" s="57">
-        <v>11.6</v>
-      </c>
-      <c r="F14" s="57">
-        <v>5.5</v>
-      </c>
-      <c r="G14" s="57">
-        <v>8.1999999999999993</v>
-      </c>
-      <c r="H14" s="56">
-        <v>7.3</v>
-      </c>
-      <c r="I14" s="55">
-        <v>1.9</v>
-      </c>
-      <c r="J14" s="55">
-        <v>1.3</v>
-      </c>
-      <c r="K14" s="55">
-        <v>27.7</v>
-      </c>
-      <c r="L14" s="55">
-        <v>8</v>
-      </c>
-      <c r="M14" s="55">
-        <v>19.600000000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="51" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15" s="57">
-        <v>13.2</v>
-      </c>
-      <c r="C15" s="57">
-        <v>15.2</v>
-      </c>
-      <c r="D15" s="57">
-        <v>26.5</v>
-      </c>
-      <c r="E15" s="57">
-        <v>15.5</v>
-      </c>
-      <c r="F15" s="57">
-        <v>25.4</v>
-      </c>
-      <c r="G15" s="57">
-        <v>16.899999999999999</v>
-      </c>
-      <c r="H15" s="56">
-        <v>9.1</v>
-      </c>
-      <c r="I15" s="55">
-        <v>17.3</v>
-      </c>
-      <c r="J15" s="55">
-        <v>4.5</v>
-      </c>
-      <c r="K15" s="55">
-        <v>20.8</v>
-      </c>
-      <c r="L15" s="55">
-        <v>3.8</v>
-      </c>
-      <c r="M15" s="55">
-        <v>6.3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="53" t="s">
-        <v>28</v>
-      </c>
-      <c r="B16" s="57">
-        <v>6.1</v>
-      </c>
-      <c r="C16" s="57">
-        <v>11</v>
-      </c>
-      <c r="D16" s="57">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="E16" s="57">
-        <v>8.3000000000000007</v>
-      </c>
-      <c r="F16" s="57">
-        <v>10.1</v>
-      </c>
-      <c r="G16" s="57">
-        <v>10.3</v>
-      </c>
-      <c r="H16" s="56">
-        <v>14.2</v>
-      </c>
-      <c r="I16" s="55">
-        <v>15</v>
-      </c>
-      <c r="J16" s="55">
-        <v>9.9</v>
-      </c>
-      <c r="K16" s="55">
-        <v>8.9</v>
-      </c>
-      <c r="L16" s="55">
-        <v>5.8</v>
-      </c>
-      <c r="M16" s="55">
-        <v>6.5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="51" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" s="57">
-        <v>0.6</v>
-      </c>
-      <c r="C17" s="57">
-        <v>0.5</v>
-      </c>
-      <c r="D17" s="57">
-        <v>2.6</v>
-      </c>
-      <c r="E17" s="57">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="F17" s="57">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="G17" s="57">
-        <v>0.3</v>
-      </c>
-      <c r="H17" s="56" t="s">
-        <v>18</v>
-      </c>
-      <c r="I17" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="J17" s="55">
-        <v>1.2</v>
-      </c>
-      <c r="K17" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="L17" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="M17" s="55" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="53" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="57">
-        <v>67.400000000000006</v>
-      </c>
-      <c r="C18" s="57">
-        <v>51.9</v>
-      </c>
-      <c r="D18" s="57">
-        <v>93.6</v>
-      </c>
-      <c r="E18" s="57">
-        <v>67.099999999999994</v>
-      </c>
-      <c r="F18" s="57">
-        <v>101.5</v>
-      </c>
-      <c r="G18" s="57">
-        <v>71</v>
-      </c>
-      <c r="H18" s="56">
-        <v>70.099999999999994</v>
-      </c>
-      <c r="I18" s="55">
-        <v>64.3</v>
-      </c>
-      <c r="J18" s="55">
-        <v>72</v>
-      </c>
-      <c r="K18" s="55">
-        <v>57.2</v>
-      </c>
-      <c r="L18" s="55">
-        <v>47.9</v>
-      </c>
-      <c r="M18" s="55">
-        <v>53.7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" ht="55.5" x14ac:dyDescent="0.2">
-      <c r="A19" s="64" t="s">
-        <v>31</v>
       </c>
       <c r="B19" s="65">
         <f>SUM(B14:B18)</f>
-        <v>97.5</v>
+        <v>99.399999999999991</v>
       </c>
       <c r="C19" s="65">
         <f t="shared" ref="C19:M19" si="1">SUM(C14:C18)</f>
-        <v>81.8</v>
+        <v>73.400000000000006</v>
       </c>
       <c r="D19" s="65">
         <f t="shared" si="1"/>
-        <v>132.5</v>
+        <v>171.5</v>
       </c>
       <c r="E19" s="65">
         <f t="shared" si="1"/>
-        <v>103.6</v>
+        <v>106.5</v>
       </c>
       <c r="F19" s="65">
         <f t="shared" si="1"/>
-        <v>146.6</v>
+        <v>83</v>
       </c>
       <c r="G19" s="65">
         <f t="shared" si="1"/>
-        <v>106.69999999999999</v>
+        <v>84</v>
       </c>
       <c r="H19" s="66">
         <f t="shared" si="1"/>
-        <v>100.69999999999999</v>
-      </c>
-      <c r="I19" s="66">
-        <f t="shared" si="1"/>
-        <v>98.5</v>
-      </c>
-      <c r="J19" s="66">
-        <f t="shared" si="1"/>
-        <v>88.9</v>
-      </c>
-      <c r="K19" s="66">
-        <f t="shared" si="1"/>
-        <v>114.6</v>
-      </c>
-      <c r="L19" s="66">
-        <f t="shared" si="1"/>
-        <v>65.5</v>
-      </c>
-      <c r="M19" s="66">
-        <f t="shared" si="1"/>
-        <v>86.100000000000009</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="I19" s="66"/>
+      <c r="J19" s="66"/>
+      <c r="K19" s="66"/>
+      <c r="L19" s="66"/>
+      <c r="M19" s="66"/>
     </row>
-    <row r="20" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" ht="25.5" customHeight="1">
       <c r="A20" s="8" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" ht="25.5" customHeight="1">
       <c r="A21" s="8" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" ht="24.75" customHeight="1">
       <c r="A22" s="8" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -4144,7 +3888,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0A36A47-2CCC-405A-A8E4-43645651B567}">
   <dimension ref="A1:M9"/>
-  <sheetFormatPr defaultRowHeight="24" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="24"/>
   <cols>
     <col min="1" max="1" width="35.7109375" style="4" customWidth="1"/>
     <col min="2" max="9" width="9.5703125" style="4" bestFit="1" customWidth="1"/>
@@ -4153,27 +3897,27 @@
     <col min="15" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="92" t="s">
+    <row r="1" spans="1:13">
+      <c r="A1" s="87" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="91" t="s">
-        <v>35</v>
-      </c>
-      <c r="C1" s="91"/>
-      <c r="D1" s="91"/>
-      <c r="E1" s="91"/>
-      <c r="F1" s="91"/>
-      <c r="G1" s="91"/>
-      <c r="H1" s="91"/>
-      <c r="I1" s="91"/>
-      <c r="J1" s="91"/>
-      <c r="K1" s="91"/>
-      <c r="L1" s="91"/>
-      <c r="M1" s="91"/>
+      <c r="B1" s="86" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86"/>
+      <c r="E1" s="86"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="86"/>
+      <c r="H1" s="86"/>
+      <c r="I1" s="86"/>
+      <c r="J1" s="86"/>
+      <c r="K1" s="86"/>
+      <c r="L1" s="86"/>
+      <c r="M1" s="86"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="93"/>
+    <row r="2" spans="1:13">
+      <c r="A2" s="88"/>
       <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
@@ -4196,28 +3940,28 @@
         <v>9</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:13">
       <c r="A3" s="40" t="s">
         <v>36</v>
       </c>
       <c r="B3" s="1">
         <f>'ปริมาณขยะรายเดือน '!$B$4</f>
-        <v>370.6</v>
+        <v>351.8</v>
       </c>
       <c r="C3" s="1">
         <v>336.1</v>
@@ -4227,48 +3971,48 @@
       </c>
       <c r="E3" s="1">
         <f>'ปริมาณขยะรายเดือน '!E4</f>
-        <v>359.8</v>
+        <v>405</v>
       </c>
       <c r="F3" s="1">
         <f>'ปริมาณขยะรายเดือน '!F4</f>
-        <v>411.4</v>
+        <v>450</v>
       </c>
       <c r="G3" s="1">
         <f>'ปริมาณขยะรายเดือน '!G4</f>
-        <v>420.9</v>
+        <v>465</v>
       </c>
       <c r="H3" s="1">
         <f>'ปริมาณขยะรายเดือน '!H4</f>
-        <v>359.4</v>
+        <v>480</v>
       </c>
       <c r="I3" s="1">
         <f>'ปริมาณขยะรายเดือน '!I4</f>
-        <v>365.6</v>
+        <v>0</v>
       </c>
       <c r="J3" s="1">
         <f>'ปริมาณขยะรายเดือน '!J4</f>
-        <v>350.8</v>
+        <v>0</v>
       </c>
       <c r="K3" s="1">
         <f>'ปริมาณขยะรายเดือน '!K4</f>
-        <v>341.8</v>
+        <v>0</v>
       </c>
       <c r="L3" s="1">
         <f>'ปริมาณขยะรายเดือน '!L4</f>
-        <v>349.8</v>
+        <v>0</v>
       </c>
       <c r="M3" s="1">
         <f>'ปริมาณขยะรายเดือน '!M4</f>
-        <v>331.3</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:13" ht="22.5" customHeight="1">
       <c r="A4" s="41" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B4" s="1">
         <f>'ปริมาณขยะรายเดือน '!$B$12</f>
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="C4" s="1">
         <v>0.3</v>
@@ -4278,19 +4022,19 @@
       </c>
       <c r="E4" s="1">
         <f>'ปริมาณขยะรายเดือน '!E12</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F4" s="1">
         <f>'ปริมาณขยะรายเดือน '!F12</f>
-        <v>4.7</v>
+        <v>3</v>
       </c>
       <c r="G4" s="1">
         <f>'ปริมาณขยะรายเดือน '!G12</f>
-        <v>10.8</v>
+        <v>16</v>
       </c>
       <c r="H4" s="1">
         <f>'ปริมาณขยะรายเดือน '!H12</f>
-        <v>1.9</v>
+        <v>4</v>
       </c>
       <c r="I4" s="1">
         <f>'ปริมาณขยะรายเดือน '!I12</f>
@@ -4298,11 +4042,11 @@
       </c>
       <c r="J4" s="1">
         <f>'ปริมาณขยะรายเดือน '!J12</f>
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="K4" s="1">
         <f>'ปริมาณขยะรายเดือน '!K12</f>
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="L4" s="1">
         <f>'ปริมาณขยะรายเดือน '!L12</f>
@@ -4313,13 +4057,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:13">
       <c r="A5" s="42" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B5" s="5">
         <f>'ปริมาณขยะรายเดือน '!$B$19</f>
-        <v>97.5</v>
+        <v>99.399999999999991</v>
       </c>
       <c r="C5" s="5">
         <v>81.8</v>
@@ -4329,48 +4073,48 @@
       </c>
       <c r="E5" s="5">
         <f>'ปริมาณขยะรายเดือน '!E19</f>
-        <v>103.6</v>
+        <v>106.5</v>
       </c>
       <c r="F5" s="5">
         <f>'ปริมาณขยะรายเดือน '!F19</f>
-        <v>146.6</v>
+        <v>83</v>
       </c>
       <c r="G5" s="5">
         <f>'ปริมาณขยะรายเดือน '!G19</f>
-        <v>106.69999999999999</v>
+        <v>84</v>
       </c>
       <c r="H5" s="5">
         <f>'ปริมาณขยะรายเดือน '!H19</f>
-        <v>100.69999999999999</v>
+        <v>69</v>
       </c>
       <c r="I5" s="5">
         <f>'ปริมาณขยะรายเดือน '!I19</f>
-        <v>98.5</v>
+        <v>0</v>
       </c>
       <c r="J5" s="5">
         <f>'ปริมาณขยะรายเดือน '!J19</f>
-        <v>88.9</v>
+        <v>0</v>
       </c>
       <c r="K5" s="5">
         <f>'ปริมาณขยะรายเดือน '!K19</f>
-        <v>114.6</v>
+        <v>0</v>
       </c>
       <c r="L5" s="5">
         <f>'ปริมาณขยะรายเดือน '!L19</f>
-        <v>65.5</v>
+        <v>0</v>
       </c>
       <c r="M5" s="5">
         <f>'ปริมาณขยะรายเดือน '!M19</f>
-        <v>86.100000000000009</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:13" ht="25.5" customHeight="1">
       <c r="A6" s="6" t="s">
         <v>37</v>
       </c>
       <c r="B6" s="5">
         <f>SUM(B3:B5)</f>
-        <v>468.1</v>
+        <v>452.4</v>
       </c>
       <c r="C6" s="5">
         <f t="shared" ref="C6:M6" si="0">SUM(C3:C5)</f>
@@ -4382,48 +4126,48 @@
       </c>
       <c r="E6" s="5">
         <f t="shared" si="0"/>
-        <v>463.4</v>
+        <v>512</v>
       </c>
       <c r="F6" s="5">
         <f t="shared" si="0"/>
-        <v>562.69999999999993</v>
+        <v>536</v>
       </c>
       <c r="G6" s="5">
         <f t="shared" si="0"/>
-        <v>538.4</v>
+        <v>565</v>
       </c>
       <c r="H6" s="5">
         <f t="shared" si="0"/>
-        <v>461.99999999999994</v>
+        <v>553</v>
       </c>
       <c r="I6" s="5">
         <f t="shared" si="0"/>
-        <v>464.1</v>
+        <v>0</v>
       </c>
       <c r="J6" s="5">
         <f t="shared" si="0"/>
-        <v>440.9</v>
+        <v>0</v>
       </c>
       <c r="K6" s="5">
         <f t="shared" si="0"/>
-        <v>458.9</v>
+        <v>0</v>
       </c>
       <c r="L6" s="5">
         <f t="shared" si="0"/>
-        <v>415.3</v>
+        <v>0</v>
       </c>
       <c r="M6" s="5">
         <f t="shared" si="0"/>
-        <v>417.40000000000003</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:13" ht="26.25" customHeight="1">
       <c r="A7" s="45" t="s">
         <v>38</v>
       </c>
       <c r="B7" s="43">
         <f>B5/B6</f>
-        <v>0.20828882717368083</v>
+        <v>0.21971706454465073</v>
       </c>
       <c r="C7" s="43">
         <f t="shared" ref="C7:M7" si="1">C5/C6</f>
@@ -4435,48 +4179,48 @@
       </c>
       <c r="E7" s="43">
         <f t="shared" si="1"/>
-        <v>0.22356495468277945</v>
+        <v>0.2080078125</v>
       </c>
       <c r="F7" s="43">
         <f t="shared" si="1"/>
-        <v>0.26052958947929628</v>
+        <v>0.15485074626865672</v>
       </c>
       <c r="G7" s="43">
         <f t="shared" si="1"/>
-        <v>0.19817979197622584</v>
+        <v>0.14867256637168141</v>
       </c>
       <c r="H7" s="43">
         <f t="shared" si="1"/>
-        <v>0.21796536796536797</v>
-      </c>
-      <c r="I7" s="43">
+        <v>0.12477396021699819</v>
+      </c>
+      <c r="I7" s="43" t="e">
         <f t="shared" si="1"/>
-        <v>0.21223874165050635</v>
-      </c>
-      <c r="J7" s="43">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J7" s="43" t="e">
         <f t="shared" si="1"/>
-        <v>0.20163302336130645</v>
-      </c>
-      <c r="K7" s="43">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="K7" s="43" t="e">
         <f t="shared" si="1"/>
-        <v>0.24972760950098061</v>
-      </c>
-      <c r="L7" s="43">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="L7" s="43" t="e">
         <f t="shared" si="1"/>
-        <v>0.15771731278593787</v>
-      </c>
-      <c r="M7" s="43">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="M7" s="43" t="e">
         <f t="shared" si="1"/>
-        <v>0.20627695256348827</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:13" ht="26.25" customHeight="1">
       <c r="A8" s="46" t="s">
         <v>39</v>
       </c>
       <c r="B8" s="7">
         <f>B3/B6</f>
-        <v>0.7917111728263192</v>
+        <v>0.77763041556145007</v>
       </c>
       <c r="C8" s="7">
         <f t="shared" ref="C8:M8" si="2">C3/C6</f>
@@ -4488,48 +4232,48 @@
       </c>
       <c r="E8" s="7">
         <f t="shared" si="2"/>
-        <v>0.77643504531722063</v>
+        <v>0.791015625</v>
       </c>
       <c r="F8" s="7">
         <f t="shared" si="2"/>
-        <v>0.73111782477341392</v>
+        <v>0.83955223880597019</v>
       </c>
       <c r="G8" s="7">
         <f t="shared" si="2"/>
-        <v>0.78176077265973254</v>
+        <v>0.82300884955752207</v>
       </c>
       <c r="H8" s="7">
         <f t="shared" si="2"/>
-        <v>0.77792207792207801</v>
-      </c>
-      <c r="I8" s="7">
+        <v>0.86799276672694392</v>
+      </c>
+      <c r="I8" s="7" t="e">
         <f t="shared" si="2"/>
-        <v>0.78776125834949362</v>
-      </c>
-      <c r="J8" s="7">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J8" s="7" t="e">
         <f t="shared" si="2"/>
-        <v>0.79564527103651628</v>
-      </c>
-      <c r="K8" s="7">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="K8" s="7" t="e">
         <f t="shared" si="2"/>
-        <v>0.74482458051863154</v>
-      </c>
-      <c r="L8" s="7">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="L8" s="7" t="e">
         <f t="shared" si="2"/>
-        <v>0.84228268721406208</v>
-      </c>
-      <c r="M8" s="7">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="M8" s="7" t="e">
         <f t="shared" si="2"/>
-        <v>0.79372304743651168</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:13">
       <c r="A9" s="47" t="s">
         <v>40</v>
       </c>
       <c r="B9" s="44">
         <f>B4/B6</f>
-        <v>0</v>
+        <v>2.6525198938992041E-3</v>
       </c>
       <c r="C9" s="44">
         <f t="shared" ref="C9:M9" si="3">C4/C6</f>
@@ -4541,39 +4285,39 @@
       </c>
       <c r="E9" s="44">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>9.765625E-4</v>
       </c>
       <c r="F9" s="44">
         <f t="shared" si="3"/>
-        <v>8.3525857472898542E-3</v>
+        <v>5.597014925373134E-3</v>
       </c>
       <c r="G9" s="44">
         <f t="shared" si="3"/>
-        <v>2.0059435364041606E-2</v>
+        <v>2.831858407079646E-2</v>
       </c>
       <c r="H9" s="44">
         <f t="shared" si="3"/>
-        <v>4.1125541125541128E-3</v>
-      </c>
-      <c r="I9" s="44">
+        <v>7.2332730560578659E-3</v>
+      </c>
+      <c r="I9" s="44" t="e">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J9" s="44">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J9" s="44" t="e">
         <f t="shared" si="3"/>
-        <v>2.7217056021773644E-3</v>
-      </c>
-      <c r="K9" s="44">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="K9" s="44" t="e">
         <f t="shared" si="3"/>
-        <v>5.4478099803878842E-3</v>
-      </c>
-      <c r="L9" s="44">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="L9" s="44" t="e">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="M9" s="44">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="M9" s="44" t="e">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
   </sheetData>
@@ -4591,7 +4335,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{691AF8B7-D31E-4D05-973E-8463671DFBA7}">
   <dimension ref="A1:AA24"/>
-  <sheetFormatPr defaultRowHeight="27.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="27.75"/>
   <cols>
     <col min="1" max="1" width="39.42578125" style="8" customWidth="1"/>
     <col min="2" max="13" width="8.28515625" style="9" customWidth="1"/>
@@ -4602,12 +4346,12 @@
     <col min="28" max="16384" width="9.140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="55.5" x14ac:dyDescent="0.2">
-      <c r="O1" s="74" t="s">
+    <row r="1" spans="1:27" ht="55.5">
+      <c r="O1" s="73" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:27" ht="41.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:27" ht="41.25" customHeight="1">
       <c r="B2" s="8"/>
       <c r="L2" s="9" t="s">
         <v>0</v>
@@ -4621,47 +4365,47 @@
       <c r="R2" s="10"/>
       <c r="S2" s="10"/>
     </row>
-    <row r="3" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="82"/>
-      <c r="B3" s="83"/>
-      <c r="C3" s="83"/>
-      <c r="D3" s="83"/>
-      <c r="E3" s="83"/>
-      <c r="F3" s="83"/>
-      <c r="G3" s="83"/>
-      <c r="H3" s="83"/>
-      <c r="I3" s="83"/>
-      <c r="J3" s="83"/>
-      <c r="K3" s="83"/>
-      <c r="L3" s="83"/>
-      <c r="M3" s="84"/>
+    <row r="3" spans="1:27" ht="36" customHeight="1">
+      <c r="A3" s="89"/>
+      <c r="B3" s="90"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="90"/>
+      <c r="K3" s="90"/>
+      <c r="L3" s="90"/>
+      <c r="M3" s="91"/>
       <c r="O3" s="8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:27">
       <c r="A4" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="82" t="s">
-        <v>50</v>
-      </c>
-      <c r="C4" s="83"/>
-      <c r="D4" s="83"/>
-      <c r="E4" s="83"/>
-      <c r="F4" s="83"/>
-      <c r="G4" s="83"/>
-      <c r="H4" s="83"/>
-      <c r="I4" s="83"/>
-      <c r="J4" s="83"/>
-      <c r="K4" s="83"/>
-      <c r="L4" s="83"/>
-      <c r="M4" s="84"/>
+      <c r="B4" s="89" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="90"/>
+      <c r="D4" s="90"/>
+      <c r="E4" s="90"/>
+      <c r="F4" s="90"/>
+      <c r="G4" s="90"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="90"/>
+      <c r="J4" s="90"/>
+      <c r="K4" s="90"/>
+      <c r="L4" s="90"/>
+      <c r="M4" s="91"/>
       <c r="O4" s="13" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:27" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:27" ht="21" customHeight="1">
       <c r="A5" s="14"/>
       <c r="B5" s="15" t="s">
         <v>3</v>
@@ -4685,41 +4429,41 @@
         <v>9</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="M5" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="O5" s="85" t="s">
+        <v>35</v>
+      </c>
+      <c r="O5" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="P5" s="87" t="s">
-        <v>2</v>
-      </c>
-      <c r="Q5" s="87"/>
-      <c r="R5" s="87"/>
-      <c r="S5" s="87"/>
-      <c r="T5" s="87"/>
-      <c r="U5" s="87"/>
-      <c r="V5" s="87"/>
-      <c r="W5" s="87"/>
-      <c r="X5" s="87"/>
-      <c r="Y5" s="87"/>
-      <c r="Z5" s="87"/>
-      <c r="AA5" s="87"/>
+      <c r="P5" s="92" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q5" s="92"/>
+      <c r="R5" s="92"/>
+      <c r="S5" s="92"/>
+      <c r="T5" s="92"/>
+      <c r="U5" s="92"/>
+      <c r="V5" s="92"/>
+      <c r="W5" s="92"/>
+      <c r="X5" s="92"/>
+      <c r="Y5" s="92"/>
+      <c r="Z5" s="92"/>
+      <c r="AA5" s="92"/>
     </row>
-    <row r="6" spans="1:27" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:27" ht="23.25" customHeight="1">
       <c r="A6" s="16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B6" s="60">
         <v>370.6</v>
@@ -4757,11 +4501,11 @@
       <c r="M6" s="62">
         <v>331.3</v>
       </c>
-      <c r="N6" s="81">
+      <c r="N6" s="80">
         <f>SUM(B6:M6)</f>
         <v>4381.0000000000009</v>
       </c>
-      <c r="O6" s="86"/>
+      <c r="O6" s="85"/>
       <c r="P6" s="17" t="s">
         <v>3</v>
       </c>
@@ -4784,24 +4528,24 @@
         <v>9</v>
       </c>
       <c r="W6" s="17" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="X6" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="Y6" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z6" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA6" s="17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" ht="23.25" customHeight="1">
+      <c r="A7" s="75" t="s">
         <v>11</v>
-      </c>
-      <c r="Y6" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z6" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="AA6" s="17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:27" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="76" t="s">
-        <v>16</v>
       </c>
       <c r="B7" s="18"/>
       <c r="C7" s="15"/>
@@ -4855,21 +4599,21 @@
         <v>331.3</v>
       </c>
     </row>
-    <row r="8" spans="1:27" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:27" ht="23.25" customHeight="1">
       <c r="A8" s="19" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B8" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C8" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D8" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E8" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F8" s="57">
         <v>3.5</v>
@@ -4878,25 +4622,25 @@
         <v>9.5</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="J8" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K8" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="L8" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="M8" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="O8" s="72" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="P8" s="70">
         <f>B14</f>
@@ -4936,48 +4680,48 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:27" ht="23.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:27" ht="23.25" customHeight="1">
       <c r="A9" s="19" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B9" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C9" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D9" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E9" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F9" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G9" s="57">
         <v>0.5</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="I9" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="J9" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K9" s="55">
         <v>2.5</v>
       </c>
       <c r="L9" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="M9" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="P9" s="35">
         <f>B21</f>
@@ -5028,45 +4772,45 @@
         <v>86.100000000000009</v>
       </c>
     </row>
-    <row r="10" spans="1:27" ht="23.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:27" ht="23.25" customHeight="1">
       <c r="A10" s="21" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B10" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C10" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D10" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E10" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F10" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G10" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="H10" s="15">
         <v>0.7</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="J10" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K10" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="L10" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="M10" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="O10" s="36" t="s">
         <v>37</v>
@@ -5120,45 +4864,45 @@
         <v>417.40000000000003</v>
       </c>
     </row>
-    <row r="11" spans="1:27" ht="23.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:27" ht="23.25" customHeight="1">
       <c r="A11" s="21" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B11" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C11" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D11" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E11" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F11" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G11" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="H11" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="I11" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="J11" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K11" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="L11" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="M11" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="O11" s="36"/>
       <c r="P11" s="22"/>
@@ -5174,21 +4918,21 @@
       <c r="Z11" s="20"/>
       <c r="AA11" s="20"/>
     </row>
-    <row r="12" spans="1:27" ht="23.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:27" ht="23.25" customHeight="1">
       <c r="A12" s="23" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B12" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C12" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D12" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E12" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F12" s="57">
         <v>1.2</v>
@@ -5200,19 +4944,19 @@
         <v>1.2</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="J12" s="15">
         <v>1.2</v>
       </c>
       <c r="K12" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="L12" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="M12" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="O12" s="37" t="s">
         <v>38</v>
@@ -5266,9 +5010,9 @@
         <v>0.20627695256348827</v>
       </c>
     </row>
-    <row r="13" spans="1:27" ht="23.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:27" ht="23.25" customHeight="1">
       <c r="A13" s="23" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B13" s="57">
         <v>0.8</v>
@@ -5280,31 +5024,31 @@
         <v>0.3</v>
       </c>
       <c r="E13" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F13" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G13" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="H13" s="57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="I13" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="J13" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K13" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="L13" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="M13" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="O13" s="37" t="s">
         <v>39</v>
@@ -5358,9 +5102,9 @@
         <v>0.79372304743651168</v>
       </c>
     </row>
-    <row r="14" spans="1:27" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="75" t="s">
-        <v>24</v>
+    <row r="14" spans="1:27" ht="23.25" customHeight="1">
+      <c r="A14" s="74" t="s">
+        <v>19</v>
       </c>
       <c r="B14" s="70">
         <f t="shared" ref="B14:M14" si="4">SUM(B8:B13)</f>
@@ -5411,7 +5155,7 @@
         <v>0</v>
       </c>
       <c r="O14" s="21" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="P14" s="32">
         <f t="shared" ref="P14:AA14" si="5">P8/P10</f>
@@ -5462,9 +5206,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:27" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:27" ht="23.25" customHeight="1">
       <c r="A15" s="25" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B15" s="26"/>
       <c r="C15" s="15"/>
@@ -5492,9 +5236,9 @@
       <c r="Z15" s="24"/>
       <c r="AA15" s="24"/>
     </row>
-    <row r="16" spans="1:27" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:27" ht="23.25" customHeight="1">
       <c r="A16" s="23" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B16" s="57">
         <v>10.199999999999999</v>
@@ -5533,9 +5277,9 @@
         <v>19.600000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" ht="23.25" customHeight="1">
       <c r="A17" s="23" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B17" s="57">
         <v>13.2</v>
@@ -5574,9 +5318,9 @@
         <v>6.3</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" ht="23.25" customHeight="1">
       <c r="A18" s="27" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B18" s="57">
         <v>6.1</v>
@@ -5615,9 +5359,9 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" ht="23.25" customHeight="1">
       <c r="A19" s="23" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="B19" s="57">
         <v>0.6</v>
@@ -5638,27 +5382,27 @@
         <v>0.3</v>
       </c>
       <c r="H19" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="I19" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="J19" s="15">
         <v>1.2</v>
       </c>
       <c r="K19" s="55" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="L19" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="M19" s="15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" ht="23.25" customHeight="1">
       <c r="A20" s="27" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B20" s="57">
         <v>67.400000000000006</v>
@@ -5697,9 +5441,9 @@
         <v>53.7</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13">
       <c r="A21" s="31" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B21" s="28">
         <f>SUM(B16:B20)</f>
@@ -5750,19 +5494,19 @@
         <v>86.100000000000009</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13">
       <c r="A22" s="8" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13">
       <c r="A23" s="8" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13">
       <c r="A24" s="8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -6051,38 +5795,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{222CA3C6-7107-4FBD-B9DD-2ACBBAD30DFC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="7b8fd10d-82db-4106-8c5b-83cd3e4ad2c7"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{222CA3C6-7107-4FBD-B9DD-2ACBBAD30DFC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F618D6E6-23F1-4C41-8F35-1E97B73F8E6E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="7b8fd10d-82db-4106-8c5b-83cd3e4ad2c7"/>
-    <ds:schemaRef ds:uri="abcb2651-95fa-414f-a10c-971ab93c7c80"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F618D6E6-23F1-4C41-8F35-1E97B73F8E6E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B91B40D1-58AE-4087-8790-6A4EE4537AF4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B91B40D1-58AE-4087-8790-6A4EE4537AF4}"/>
 </file>
</xml_diff>